<commit_message>
excel_to_json and update_comments_from_json works
</commit_message>
<xml_diff>
--- a/static/demo_data/Standardized example sheets/Field sampling (internal).xlsx
+++ b/static/demo_data/Standardized example sheets/Field sampling (internal).xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\glj523\Documents\github repoes\upload_web_app\static\example_sheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\glj523\Documents\github repoes\upload_web_app\static\demo_data\Standardized example sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DAB1227-3708-4AEC-9CDB-45A8E1677EED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{913BA8A6-6A19-4EA9-9EFC-62DD3908381D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{F20BE04D-14A6-4DFA-9322-DA461E992517}"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{F20BE04D-14A6-4DFA-9322-DA461E992517}"/>
   </bookViews>
   <sheets>
     <sheet name="eDNA_Archive_sampling_(20231027" sheetId="2" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="125">
   <si>
     <t>Expected column names and positions:</t>
   </si>
@@ -92,9 +92,6 @@
   </si>
   <si>
     <t>decimal degrees, max 2 digits, max 8 decimal points (-180 to 180)</t>
-  </si>
-  <si>
-    <t>Examples of accepted data:</t>
   </si>
   <si>
     <t>*If a column is required, this means that the sheet will be rejected if there are any values missing from that column</t>
@@ -442,6 +439,9 @@
   </si>
   <si>
     <t>&lt;measurement/observation type&gt;: &lt;measurement/observation&gt; &lt;unit (optional)&gt;</t>
+  </si>
+  <si>
+    <t>Examples data:</t>
   </si>
 </sst>
 </file>
@@ -711,9 +711,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -751,7 +751,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -857,7 +857,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -999,7 +999,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1081,123 +1081,123 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="L1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="P1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="S1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="L1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="P1" s="1" t="s">
+      <c r="U1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AB1" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="Q1" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="Y1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="AD1" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="AE1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="AG1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="AD1" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:35" s="18" customFormat="1" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>9</v>
+        <v>124</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G2" s="19">
         <v>61.139899999999997</v>
@@ -1206,28 +1206,28 @@
         <v>-45.534700000000001</v>
       </c>
       <c r="I2" s="18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J2" s="18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K2" s="18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="L2" s="18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="M2" s="18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N2" s="18">
         <v>10</v>
       </c>
       <c r="O2" s="18" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P2" s="18" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Q2" s="18">
         <v>10</v>
@@ -1239,58 +1239,60 @@
         <v>4</v>
       </c>
       <c r="T2" s="18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="U2" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="V2" s="18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="W2" s="18" t="s">
         <v>5</v>
       </c>
       <c r="X2" s="18" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="Y2" s="18">
         <v>37</v>
       </c>
       <c r="Z2" s="18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA2" s="18" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AB2" s="18" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AC2" s="18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AD2" s="18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AE2" s="18" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AF2" s="18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:35" s="18" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="4"/>
+      <c r="A3" s="4" t="s">
+        <v>124</v>
+      </c>
       <c r="B3" s="18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G3" s="19">
         <v>61.139899999999997</v>
@@ -1299,28 +1301,28 @@
         <v>-45.534700000000001</v>
       </c>
       <c r="I3" s="18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K3" s="18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="L3" s="18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="M3" s="18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="N3" s="18">
         <v>200</v>
       </c>
       <c r="O3" s="18" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="P3" s="18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q3" s="18">
         <v>200</v>
@@ -1329,61 +1331,63 @@
         <v>200</v>
       </c>
       <c r="S3" s="18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="T3" s="18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="U3" s="19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="V3" s="18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="W3" s="18" t="s">
         <v>5</v>
       </c>
       <c r="X3" s="18" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="Y3" s="18">
         <v>37</v>
       </c>
       <c r="Z3" s="18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AA3" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AB3" s="18" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AC3" s="18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AD3" s="18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AE3" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="AF3" s="18" t="s">
         <v>79</v>
-      </c>
-      <c r="AF3" s="18" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:35" s="18" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="4"/>
+      <c r="A4" s="4" t="s">
+        <v>124</v>
+      </c>
       <c r="B4" s="18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G4" s="19">
         <v>61.139899999999997</v>
@@ -1392,324 +1396,324 @@
         <v>-45.534700000000001</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J4" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="K4" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="K4" s="18" t="s">
-        <v>65</v>
-      </c>
       <c r="L4" s="18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="M4" s="18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="N4" s="18" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="O4" s="18" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="P4" s="18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="Q4" s="18" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="R4" s="18" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="S4" s="18" t="s">
         <v>6</v>
       </c>
       <c r="T4" s="18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="U4" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="V4" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="W4" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="X4" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="Y4" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="Z4" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="AA4" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="AB4" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="AC4" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="AD4" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="AE4" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="AF4" s="18" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="1:35" s="6" customFormat="1" ht="81.599999999999994" x14ac:dyDescent="0.3">
+      <c r="A5" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="O5" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="U5" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="X5" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="Z5" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="AA5" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="AB5" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="AC5" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="AD5" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="AE5" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="AF5" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="AG5" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="AH5" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="AI5" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="6" spans="1:35" s="5" customFormat="1" ht="61.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="D6" s="8"/>
+      <c r="E6" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="H6" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="V4" s="18" t="s">
-        <v>69</v>
-      </c>
-      <c r="W4" s="18" t="s">
-        <v>70</v>
-      </c>
-      <c r="X4" s="18" t="s">
-        <v>105</v>
-      </c>
-      <c r="Y4" s="18" t="s">
-        <v>119</v>
-      </c>
-      <c r="Z4" s="18" t="s">
-        <v>82</v>
-      </c>
-      <c r="AA4" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="AB4" s="18" t="s">
-        <v>88</v>
-      </c>
-      <c r="AC4" s="18" t="s">
-        <v>103</v>
-      </c>
-      <c r="AD4" s="18" t="s">
-        <v>103</v>
-      </c>
-      <c r="AE4" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="AF4" s="18" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="6" spans="1:35" s="6" customFormat="1" ht="81.599999999999994" x14ac:dyDescent="0.3">
-      <c r="A6" s="16" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5" t="s">
+      <c r="I6" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="J6" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="K6" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="L6" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="M6" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="N6" s="5" t="s">
+      <c r="L6" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="M6" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="N6" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="O6" s="20" t="s">
-        <v>106</v>
+      <c r="O6" s="12" t="s">
+        <v>55</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="S6" s="5" t="s">
-        <v>11</v>
+        <v>56</v>
+      </c>
+      <c r="S6" s="12" t="s">
+        <v>58</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>104</v>
+        <v>121</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="V6" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="W6" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="X6" s="20" t="s">
-        <v>106</v>
+        <v>40</v>
+      </c>
+      <c r="X6" s="5" t="s">
+        <v>70</v>
       </c>
       <c r="Y6" s="5" t="s">
         <v>72</v>
       </c>
       <c r="Z6" s="5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="AA6" s="5" t="s">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="AB6" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="AC6" s="5" t="s">
-        <v>102</v>
+        <v>85</v>
+      </c>
+      <c r="AC6" s="13" t="s">
+        <v>88</v>
       </c>
       <c r="AD6" s="5" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="AE6" s="5" t="s">
-        <v>124</v>
+        <v>73</v>
       </c>
       <c r="AF6" s="5" t="s">
-        <v>124</v>
+        <v>75</v>
       </c>
       <c r="AG6" s="5" t="s">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="AH6" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="AI6" s="5" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:35" s="5" customFormat="1" ht="61.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="L7" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="M7" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="N7" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="O7" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="P7" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="Q7" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="R7" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="S7" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="T7" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="U7" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="X7" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="Y7" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="Z7" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="AA7" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="AB7" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="AC7" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="AD7" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="AE7" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="AF7" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="AG7" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="AH7" s="5" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="8" spans="1:35" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="17" t="s">
+    <row r="7" spans="1:35" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="H7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="I7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="J8" s="6" t="s">
+      <c r="J7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="K8" s="6" t="s">
+      <c r="K7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="L8" s="6" t="s">
+      <c r="L7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="M8" s="6" t="s">
+      <c r="M7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="P8" s="7"/>
-      <c r="Q8" s="7"/>
-      <c r="R8" s="7"/>
-      <c r="U8" s="5"/>
-      <c r="Z8" s="6" t="s">
+      <c r="P7" s="7"/>
+      <c r="Q7" s="7"/>
+      <c r="R7" s="7"/>
+      <c r="U7" s="5"/>
+      <c r="Z7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="AA8" s="6" t="s">
+      <c r="AA7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="AE8" s="6" t="s">
+      <c r="AE7" s="6" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1717,7 +1721,7 @@
     <row r="10" spans="1:35" s="17" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="1:35" s="17" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>